<commit_message>
Remove stale shared-formula instructions and verify workbooks in Excel
</commit_message>
<xml_diff>
--- a/verification/registry-records.xlsx
+++ b/verification/registry-records.xlsx
@@ -2879,20 +2879,20 @@
       <x:c r="B5" s="25" t="str">
         <x:v>No Table</x:v>
       </x:c>
-      <x:c r="C5" s="22" t="n">
+      <x:c r="C5" s="22">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A5,'S0 Registry Executions'!$G$2:$G$518,B5,'S0 Registry Executions'!$M$2:$M$518,"Yes")</x:f>
         <x:v>90</x:v>
       </x:c>
-      <x:c r="D5" s="22" t="n">
+      <x:c r="D5" s="22">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A5,'S0 Registry Executions'!$G$2:$G$518,B5,'S0 Registry Executions'!$M$2:$M$518,"No")</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="E5" s="22" t="n">
-        <x:f t="shared" ref="E5:E10" si="0">C5+D5</x:f>
+      <x:c r="E5" s="22">
+        <x:f>C5+D5</x:f>
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F5" s="27" t="n">
-        <x:f t="shared" ref="F5:F10" si="1">IFERROR(D5/E5,0)</x:f>
+      <x:c r="F5" s="27">
+        <x:f>IFERROR(D5/E5,0)</x:f>
         <x:v>0.26229508196721313</x:v>
       </x:c>
       <x:c r="G5" s="24" t="str">
@@ -2912,20 +2912,20 @@
       <x:c r="B6" s="25" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="C6" s="22" t="n">
+      <x:c r="C6" s="22">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A6,'S0 Registry Executions'!$G$2:$G$518,B6,'S0 Registry Executions'!$M$2:$M$518,"Yes")</x:f>
         <x:v>90</x:v>
       </x:c>
-      <x:c r="D6" s="22" t="n">
+      <x:c r="D6" s="22">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A6,'S0 Registry Executions'!$G$2:$G$518,B6,'S0 Registry Executions'!$M$2:$M$518,"No")</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="n">
-        <x:f t="shared" si="0">C6+D6</x:f>
+      <x:c r="E6" s="22">
+        <x:f>C6+D6</x:f>
         <x:v>92</x:v>
       </x:c>
-      <x:c r="F6" s="27" t="n">
-        <x:f t="shared" si="1">IFERROR(D6/E6,0)</x:f>
+      <x:c r="F6" s="27">
+        <x:f>IFERROR(D6/E6,0)</x:f>
         <x:v>0.021739130434782608</x:v>
       </x:c>
       <x:c r="G6" s="24" t="str">
@@ -2945,20 +2945,20 @@
       <x:c r="B7" t="str">
         <x:v>No Table</x:v>
       </x:c>
-      <x:c r="C7" t="n">
+      <x:c r="C7">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A7,'S0 Registry Executions'!$G$2:$G$518,B7,'S0 Registry Executions'!$M$2:$M$518,"Yes")</x:f>
         <x:v>90</x:v>
       </x:c>
-      <x:c r="D7" t="n">
+      <x:c r="D7">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A7,'S0 Registry Executions'!$G$2:$G$518,B7,'S0 Registry Executions'!$M$2:$M$518,"No")</x:f>
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E7" t="n">
-        <x:f t="shared" si="0">C7+D7</x:f>
+      <x:c r="E7">
+        <x:f>C7+D7</x:f>
         <x:v>99</x:v>
       </x:c>
-      <x:c r="F7" s="28" t="n">
-        <x:f t="shared" si="1">IFERROR(D7/E7,0)</x:f>
+      <x:c r="F7" s="28">
+        <x:f>IFERROR(D7/E7,0)</x:f>
         <x:v>0.09090909090909091</x:v>
       </x:c>
       <x:c r="G7" s="4" t="str">
@@ -2978,20 +2978,20 @@
       <x:c r="B8" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="C8" t="n">
+      <x:c r="C8">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A8,'S0 Registry Executions'!$G$2:$G$518,B8,'S0 Registry Executions'!$M$2:$M$518,"Yes")</x:f>
         <x:v>90</x:v>
       </x:c>
-      <x:c r="D8" t="n">
+      <x:c r="D8">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A8,'S0 Registry Executions'!$G$2:$G$518,B8,'S0 Registry Executions'!$M$2:$M$518,"No")</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E8" t="n">
-        <x:f t="shared" si="0">C8+D8</x:f>
+      <x:c r="E8">
+        <x:f>C8+D8</x:f>
         <x:v>93</x:v>
       </x:c>
-      <x:c r="F8" s="28" t="n">
-        <x:f t="shared" si="1">IFERROR(D8/E8,0)</x:f>
+      <x:c r="F8" s="28">
+        <x:f>IFERROR(D8/E8,0)</x:f>
         <x:v>0.03225806451612903</x:v>
       </x:c>
       <x:c r="G8" s="4" t="str">
@@ -3011,20 +3011,20 @@
       <x:c r="B9" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="C9" t="n">
+      <x:c r="C9">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A9,'S0 Registry Executions'!$G$2:$G$518,B9,'S0 Registry Executions'!$M$2:$M$518,"Yes")</x:f>
         <x:v>90</x:v>
       </x:c>
-      <x:c r="D9" t="n">
+      <x:c r="D9">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A9,'S0 Registry Executions'!$G$2:$G$518,B9,'S0 Registry Executions'!$M$2:$M$518,"No")</x:f>
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E9" t="n">
-        <x:f t="shared" si="0">C9+D9</x:f>
+      <x:c r="E9">
+        <x:f>C9+D9</x:f>
         <x:v>101</x:v>
       </x:c>
-      <x:c r="F9" s="28" t="n">
-        <x:f t="shared" si="1">IFERROR(D9/E9,0)</x:f>
+      <x:c r="F9" s="28">
+        <x:f>IFERROR(D9/E9,0)</x:f>
         <x:v>0.10891089108910891</x:v>
       </x:c>
       <x:c r="G9" s="4" t="str">
@@ -3044,20 +3044,20 @@
       <x:c r="B10" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="C10" t="n">
+      <x:c r="C10">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A10,'S0 Registry Executions'!$G$2:$G$518,B10,'S0 Registry Executions'!$M$2:$M$518,"Yes")</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D10" t="n">
+      <x:c r="D10">
         <x:f>COUNTIFS('S0 Registry Executions'!$C$2:$C$518,A10,'S0 Registry Executions'!$G$2:$G$518,B10,'S0 Registry Executions'!$M$2:$M$518,"No")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E10" t="n">
-        <x:f t="shared" si="0">C10+D10</x:f>
+      <x:c r="E10">
+        <x:f>C10+D10</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F10" s="28" t="n">
-        <x:f t="shared" si="1">IFERROR(D10/E10,0)</x:f>
+      <x:c r="F10" s="28">
+        <x:f>IFERROR(D10/E10,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="4" t="str">
@@ -3095,19 +3095,19 @@
       <x:c r="A13" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B13" t="n">
+      <x:c r="B13">
         <x:f>SUMIFS($D$5:$D$10,$B$5:$B$10,A13,$G$5:$G$10,"Yes")</x:f>
         <x:v>41</x:v>
       </x:c>
-      <x:c r="C13" t="n">
+      <x:c r="C13">
         <x:f>SUMIFS($E$5:$E$10,$B$5:$B$10,A13,$G$5:$G$10,"Yes")</x:f>
         <x:v>221</x:v>
       </x:c>
-      <x:c r="D13" s="28" t="n">
+      <x:c r="D13" s="28">
         <x:f>IFERROR(B13/C13,0)</x:f>
         <x:v>0.18552036199095023</x:v>
       </x:c>
-      <x:c r="E13" t="n">
+      <x:c r="E13">
         <x:f>C13-B13</x:f>
         <x:v>180</x:v>
       </x:c>
@@ -3125,19 +3125,19 @@
       <x:c r="A14" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B14" t="n">
+      <x:c r="B14">
         <x:f>SUMIFS($D$5:$D$10,$B$5:$B$10,A14,$G$5:$G$10,"Yes")</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C14" t="n">
+      <x:c r="C14">
         <x:f>SUMIFS($E$5:$E$10,$B$5:$B$10,A14,$G$5:$G$10,"Yes")</x:f>
         <x:v>185</x:v>
       </x:c>
-      <x:c r="D14" s="28" t="n">
+      <x:c r="D14" s="28">
         <x:f>IFERROR(B14/C14,0)</x:f>
         <x:v>0.02702702702702703</x:v>
       </x:c>
-      <x:c r="E14" t="n">
+      <x:c r="E14">
         <x:f>C14-B14</x:f>
         <x:v>180</x:v>
       </x:c>
@@ -3172,23 +3172,23 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="n">
+      <x:c r="A18">
         <x:f>COUNTA('S0 Registry Executions'!A2:A518)</x:f>
         <x:v>517</x:v>
       </x:c>
-      <x:c r="B18" t="n">
+      <x:c r="B18">
         <x:f>COUNTIF('S0 Registry Executions'!M2:M518,"Yes")</x:f>
         <x:v>460</x:v>
       </x:c>
-      <x:c r="C18" t="n">
+      <x:c r="C18">
         <x:f>COUNTIF('S0 Registry Executions'!M2:M518,"No")</x:f>
         <x:v>57</x:v>
       </x:c>
-      <x:c r="D18" t="n">
+      <x:c r="D18">
         <x:f>COUNTIF('S0 Registry Executions'!S2:S518,"Lineage only")</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F18" t="n">
+      <x:c r="F18">
         <x:f>SUM(C13:C14)</x:f>
         <x:v>406</x:v>
       </x:c>

</xml_diff>